<commit_message>
Update dashboard with July demand data
</commit_message>
<xml_diff>
--- a/data/raw/Product List 20260629.xlsx
+++ b/data/raw/Product List 20260629.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rbioffice-my.sharepoint.com/personal/lkearney_timhortons_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rbioffice.sharepoint.com/teams/Site5/Shared Documents/TH DATA2/SHARE/RETAIL/Canada Sales/Demand Review/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{FB14448E-8070-4CB5-BCAC-353740F7ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74149B08-1AFB-4BFA-B57F-88A3FF5D84D5}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{FB14448E-8070-4CB5-BCAC-353740F7ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{003C2916-B0E9-4434-ACAB-2E044D0E8CB4}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4643,7 +4643,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -4784,9 +4784,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4824,7 +4824,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4930,7 +4930,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5072,7 +5072,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -5081,28 +5081,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4229257-8101-4DBC-97FF-A61A6AACC722}">
   <dimension ref="A1:Q412"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.6"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.140625" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.42578125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.42578125" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.140625" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="20.42578125" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="23.1796875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.81640625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.453125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="31.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.453125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="46.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.1796875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="12.7265625" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="20.453125" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="18" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.42578125" hidden="1" customWidth="1"/>
-    <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.453125" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="25.81640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="20.100000000000001">
+    <row r="1" spans="1:17" ht="20" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5119,18 +5119,18 @@
       <c r="L1" s="3"/>
       <c r="M1" s="3"/>
     </row>
-    <row r="2" spans="1:17" ht="13.5" customHeight="1">
+    <row r="2" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="1:17" ht="12.95">
+    <row r="4" spans="1:17" ht="13" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -5153,7 +5153,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="Q5" s="7"/>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>20</v>
       </c>
@@ -5257,7 +5257,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>20</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>20</v>
       </c>
@@ -5363,7 +5363,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>20</v>
       </c>
@@ -5416,7 +5416,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>20</v>
       </c>
@@ -5469,7 +5469,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
@@ -5522,7 +5522,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
@@ -5575,7 +5575,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>20</v>
       </c>
@@ -5628,7 +5628,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
@@ -5681,7 +5681,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>20</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>20</v>
       </c>
@@ -5787,7 +5787,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>20</v>
       </c>
@@ -5840,7 +5840,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>20</v>
       </c>
@@ -5893,7 +5893,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>20</v>
       </c>
@@ -5946,7 +5946,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>20</v>
       </c>
@@ -5999,7 +5999,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>20</v>
       </c>
@@ -6052,7 +6052,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>20</v>
       </c>
@@ -6105,7 +6105,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>20</v>
       </c>
@@ -6158,7 +6158,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>20</v>
       </c>
@@ -6211,7 +6211,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>20</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>20</v>
       </c>
@@ -6317,7 +6317,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>20</v>
       </c>
@@ -6370,7 +6370,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="28" spans="1:17">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>20</v>
       </c>
@@ -6423,7 +6423,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="1:17">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>20</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="30" spans="1:17">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>20</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>20</v>
       </c>
@@ -6582,7 +6582,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="32" spans="1:17">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>20</v>
       </c>
@@ -6635,7 +6635,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:17">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>20</v>
       </c>
@@ -6688,7 +6688,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="34" spans="1:17">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>20</v>
       </c>
@@ -6741,7 +6741,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="35" spans="1:17">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>20</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:17">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>20</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:17">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>20</v>
       </c>
@@ -6900,7 +6900,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:17">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>20</v>
       </c>
@@ -6953,7 +6953,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" spans="1:17">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>20</v>
       </c>
@@ -7006,7 +7006,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:17">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>20</v>
       </c>
@@ -7059,7 +7059,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="41" spans="1:17">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>20</v>
       </c>
@@ -7112,7 +7112,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="42" spans="1:17">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>20</v>
       </c>
@@ -7165,7 +7165,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="43" spans="1:17">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>20</v>
       </c>
@@ -7218,7 +7218,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="44" spans="1:17">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>20</v>
       </c>
@@ -7271,7 +7271,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="45" spans="1:17">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>20</v>
       </c>
@@ -7324,7 +7324,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="46" spans="1:17">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>20</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="47" spans="1:17">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>20</v>
       </c>
@@ -7430,7 +7430,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="48" spans="1:17">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>20</v>
       </c>
@@ -7483,7 +7483,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="49" spans="1:17">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>20</v>
       </c>
@@ -7536,7 +7536,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="50" spans="1:17">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>20</v>
       </c>
@@ -7589,7 +7589,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="51" spans="1:17">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>20</v>
       </c>
@@ -7642,7 +7642,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="52" spans="1:17">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>20</v>
       </c>
@@ -7695,7 +7695,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="53" spans="1:17">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>20</v>
       </c>
@@ -7748,7 +7748,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="54" spans="1:17">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>20</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="55" spans="1:17">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>20</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="56" spans="1:17">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>20</v>
       </c>
@@ -7907,7 +7907,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="57" spans="1:17">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>20</v>
       </c>
@@ -7960,7 +7960,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="58" spans="1:17">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>20</v>
       </c>
@@ -8013,7 +8013,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="59" spans="1:17">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>20</v>
       </c>
@@ -8066,7 +8066,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="60" spans="1:17">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>20</v>
       </c>
@@ -8119,7 +8119,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="61" spans="1:17">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>20</v>
       </c>
@@ -8172,7 +8172,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="62" spans="1:17">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>20</v>
       </c>
@@ -8225,7 +8225,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="63" spans="1:17">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>20</v>
       </c>
@@ -8278,7 +8278,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="64" spans="1:17">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>20</v>
       </c>
@@ -8331,7 +8331,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="65" spans="1:17">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>20</v>
       </c>
@@ -8384,7 +8384,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="66" spans="1:17">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>20</v>
       </c>
@@ -8437,7 +8437,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:17">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>20</v>
       </c>
@@ -8490,7 +8490,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="68" spans="1:17">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>20</v>
       </c>
@@ -8543,7 +8543,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="69" spans="1:17">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>20</v>
       </c>
@@ -8596,7 +8596,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="70" spans="1:17">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>20</v>
       </c>
@@ -8649,7 +8649,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:17">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>20</v>
       </c>
@@ -8702,7 +8702,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="72" spans="1:17">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>20</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="73" spans="1:17">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>20</v>
       </c>
@@ -8808,7 +8808,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="74" spans="1:17">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>20</v>
       </c>
@@ -8861,7 +8861,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="75" spans="1:17">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>20</v>
       </c>
@@ -8914,7 +8914,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="76" spans="1:17">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>20</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="77" spans="1:17">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>20</v>
       </c>
@@ -9020,7 +9020,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="78" spans="1:17">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>20</v>
       </c>
@@ -9073,7 +9073,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="79" spans="1:17">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>20</v>
       </c>
@@ -9126,7 +9126,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="80" spans="1:17">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>20</v>
       </c>
@@ -9179,7 +9179,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="81" spans="1:17">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>20</v>
       </c>
@@ -9232,7 +9232,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="82" spans="1:17">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>20</v>
       </c>
@@ -9285,7 +9285,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="83" spans="1:17">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>20</v>
       </c>
@@ -9338,7 +9338,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="84" spans="1:17">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>20</v>
       </c>
@@ -9391,7 +9391,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="85" spans="1:17">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="6" t="s">
         <v>20</v>
       </c>
@@ -9444,7 +9444,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="86" spans="1:17">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>20</v>
       </c>
@@ -9497,7 +9497,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="87" spans="1:17">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>20</v>
       </c>
@@ -9550,7 +9550,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="88" spans="1:17">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>20</v>
       </c>
@@ -9603,7 +9603,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="89" spans="1:17">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>20</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="90" spans="1:17">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>20</v>
       </c>
@@ -9709,7 +9709,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="91" spans="1:17">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>20</v>
       </c>
@@ -9762,7 +9762,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="92" spans="1:17">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>20</v>
       </c>
@@ -9815,7 +9815,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="93" spans="1:17">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>20</v>
       </c>
@@ -9868,7 +9868,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="94" spans="1:17">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>20</v>
       </c>
@@ -9921,7 +9921,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="95" spans="1:17">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>20</v>
       </c>
@@ -9974,7 +9974,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="96" spans="1:17">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>20</v>
       </c>
@@ -10027,7 +10027,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="97" spans="1:17">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>20</v>
       </c>
@@ -10080,7 +10080,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="98" spans="1:17">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>20</v>
       </c>
@@ -10133,7 +10133,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="99" spans="1:17">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>20</v>
       </c>
@@ -10186,7 +10186,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="100" spans="1:17">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>20</v>
       </c>
@@ -10239,7 +10239,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="101" spans="1:17">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>20</v>
       </c>
@@ -10292,7 +10292,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="102" spans="1:17">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="6" t="s">
         <v>20</v>
       </c>
@@ -10345,7 +10345,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="103" spans="1:17">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="6" t="s">
         <v>20</v>
       </c>
@@ -10398,7 +10398,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="104" spans="1:17">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="6" t="s">
         <v>20</v>
       </c>
@@ -10451,7 +10451,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="105" spans="1:17">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="6" t="s">
         <v>20</v>
       </c>
@@ -10504,7 +10504,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="106" spans="1:17">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="6" t="s">
         <v>20</v>
       </c>
@@ -10557,7 +10557,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="107" spans="1:17">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="6" t="s">
         <v>20</v>
       </c>
@@ -10610,7 +10610,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="108" spans="1:17">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="6" t="s">
         <v>20</v>
       </c>
@@ -10663,7 +10663,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="109" spans="1:17">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="6" t="s">
         <v>20</v>
       </c>
@@ -10716,7 +10716,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="110" spans="1:17">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="6" t="s">
         <v>20</v>
       </c>
@@ -10769,7 +10769,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="111" spans="1:17">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="6" t="s">
         <v>20</v>
       </c>
@@ -10822,7 +10822,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="112" spans="1:17">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="6" t="s">
         <v>20</v>
       </c>
@@ -10875,7 +10875,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="113" spans="1:17">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="6" t="s">
         <v>20</v>
       </c>
@@ -10928,7 +10928,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="114" spans="1:17">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="6" t="s">
         <v>20</v>
       </c>
@@ -10981,7 +10981,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="115" spans="1:17">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" s="6" t="s">
         <v>20</v>
       </c>
@@ -11034,7 +11034,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="116" spans="1:17">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" s="6" t="s">
         <v>20</v>
       </c>
@@ -11087,7 +11087,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="117" spans="1:17">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
         <v>20</v>
       </c>
@@ -11140,7 +11140,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="118" spans="1:17">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" s="6" t="s">
         <v>20</v>
       </c>
@@ -11193,7 +11193,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="119" spans="1:17">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" s="6" t="s">
         <v>20</v>
       </c>
@@ -11246,7 +11246,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="120" spans="1:17">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="6" t="s">
         <v>20</v>
       </c>
@@ -11299,7 +11299,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="121" spans="1:17">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="6" t="s">
         <v>20</v>
       </c>
@@ -11352,7 +11352,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="122" spans="1:17">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" s="6" t="s">
         <v>20</v>
       </c>
@@ -11405,7 +11405,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="123" spans="1:17">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" s="6" t="s">
         <v>20</v>
       </c>
@@ -11458,7 +11458,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="124" spans="1:17">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" s="6" t="s">
         <v>20</v>
       </c>
@@ -11511,7 +11511,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="125" spans="1:17">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" s="6" t="s">
         <v>20</v>
       </c>
@@ -11564,7 +11564,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="126" spans="1:17">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" s="6" t="s">
         <v>20</v>
       </c>
@@ -11617,7 +11617,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="127" spans="1:17">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="6" t="s">
         <v>20</v>
       </c>
@@ -11670,7 +11670,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="128" spans="1:17">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="6" t="s">
         <v>20</v>
       </c>
@@ -11723,7 +11723,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="129" spans="1:17">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" s="6" t="s">
         <v>20</v>
       </c>
@@ -11776,7 +11776,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="130" spans="1:17">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" s="6" t="s">
         <v>20</v>
       </c>
@@ -11829,7 +11829,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="131" spans="1:17">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" s="6" t="s">
         <v>20</v>
       </c>
@@ -11882,7 +11882,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="132" spans="1:17">
+    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" s="6" t="s">
         <v>20</v>
       </c>
@@ -11935,7 +11935,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="133" spans="1:17">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="6" t="s">
         <v>20</v>
       </c>
@@ -11988,7 +11988,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="134" spans="1:17">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="6" t="s">
         <v>20</v>
       </c>
@@ -12041,7 +12041,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="135" spans="1:17">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" s="6" t="s">
         <v>20</v>
       </c>
@@ -12094,7 +12094,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="136" spans="1:17">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" s="6" t="s">
         <v>20</v>
       </c>
@@ -12147,7 +12147,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="137" spans="1:17">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" s="6" t="s">
         <v>20</v>
       </c>
@@ -12200,7 +12200,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="138" spans="1:17">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" s="6" t="s">
         <v>20</v>
       </c>
@@ -12253,7 +12253,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="139" spans="1:17">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="6" t="s">
         <v>20</v>
       </c>
@@ -12306,7 +12306,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="140" spans="1:17">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" s="6" t="s">
         <v>20</v>
       </c>
@@ -12359,7 +12359,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="141" spans="1:17">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" s="6" t="s">
         <v>20</v>
       </c>
@@ -12412,7 +12412,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="142" spans="1:17">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" s="6" t="s">
         <v>20</v>
       </c>
@@ -12465,7 +12465,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="143" spans="1:17">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" s="6" t="s">
         <v>20</v>
       </c>
@@ -12518,7 +12518,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="144" spans="1:17">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" s="6" t="s">
         <v>20</v>
       </c>
@@ -12571,7 +12571,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="145" spans="1:17">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" s="6" t="s">
         <v>20</v>
       </c>
@@ -12624,7 +12624,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="146" spans="1:17">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" s="6" t="s">
         <v>20</v>
       </c>
@@ -12677,7 +12677,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="147" spans="1:17">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" s="6" t="s">
         <v>20</v>
       </c>
@@ -12730,7 +12730,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="148" spans="1:17">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148" s="6" t="s">
         <v>20</v>
       </c>
@@ -12783,7 +12783,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="149" spans="1:17">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A149" s="6" t="s">
         <v>20</v>
       </c>
@@ -12836,7 +12836,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="150" spans="1:17">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A150" s="6" t="s">
         <v>20</v>
       </c>
@@ -12889,7 +12889,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="151" spans="1:17">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" s="6" t="s">
         <v>20</v>
       </c>
@@ -12942,7 +12942,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="152" spans="1:17">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" s="6" t="s">
         <v>20</v>
       </c>
@@ -12995,7 +12995,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="153" spans="1:17">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153" s="6" t="s">
         <v>20</v>
       </c>
@@ -13048,7 +13048,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="154" spans="1:17">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
         <v>20</v>
       </c>
@@ -13101,7 +13101,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="155" spans="1:17">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A155" s="6" t="s">
         <v>20</v>
       </c>
@@ -13154,7 +13154,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="156" spans="1:17">
+    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A156" s="6" t="s">
         <v>20</v>
       </c>
@@ -13207,7 +13207,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="157" spans="1:17">
+    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A157" s="6" t="s">
         <v>20</v>
       </c>
@@ -13260,7 +13260,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="158" spans="1:17">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A158" s="6" t="s">
         <v>20</v>
       </c>
@@ -13313,7 +13313,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="159" spans="1:17">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159" s="6" t="s">
         <v>20</v>
       </c>
@@ -13366,7 +13366,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="160" spans="1:17">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" s="6" t="s">
         <v>20</v>
       </c>
@@ -13419,7 +13419,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="161" spans="1:17">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" s="6" t="s">
         <v>20</v>
       </c>
@@ -13472,7 +13472,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="162" spans="1:17">
+    <row r="162" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" s="6" t="s">
         <v>20</v>
       </c>
@@ -13525,7 +13525,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="163" spans="1:17">
+    <row r="163" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" s="6" t="s">
         <v>20</v>
       </c>
@@ -13578,7 +13578,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="164" spans="1:17">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" s="6" t="s">
         <v>20</v>
       </c>
@@ -13631,7 +13631,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="165" spans="1:17">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" s="6" t="s">
         <v>20</v>
       </c>
@@ -13684,7 +13684,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="166" spans="1:17">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" s="6" t="s">
         <v>20</v>
       </c>
@@ -13737,7 +13737,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="167" spans="1:17">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A167" s="6" t="s">
         <v>20</v>
       </c>
@@ -13790,7 +13790,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="168" spans="1:17">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168" s="6" t="s">
         <v>20</v>
       </c>
@@ -13843,7 +13843,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="169" spans="1:17">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169" s="6" t="s">
         <v>20</v>
       </c>
@@ -13896,7 +13896,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="170" spans="1:17">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170" s="6" t="s">
         <v>20</v>
       </c>
@@ -13949,7 +13949,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="171" spans="1:17">
+    <row r="171" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A171" s="6" t="s">
         <v>20</v>
       </c>
@@ -14002,7 +14002,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="172" spans="1:17">
+    <row r="172" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A172" s="6" t="s">
         <v>20</v>
       </c>
@@ -14055,7 +14055,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="173" spans="1:17">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A173" s="6" t="s">
         <v>20</v>
       </c>
@@ -14108,7 +14108,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="174" spans="1:17">
+    <row r="174" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A174" s="6" t="s">
         <v>20</v>
       </c>
@@ -14161,7 +14161,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="175" spans="1:17">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A175" s="6" t="s">
         <v>20</v>
       </c>
@@ -14214,7 +14214,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="176" spans="1:17">
+    <row r="176" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A176" s="6" t="s">
         <v>20</v>
       </c>
@@ -14267,7 +14267,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="177" spans="1:17">
+    <row r="177" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A177" s="6" t="s">
         <v>20</v>
       </c>
@@ -14320,7 +14320,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="178" spans="1:17">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A178" s="6" t="s">
         <v>20</v>
       </c>
@@ -14373,7 +14373,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="179" spans="1:17">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A179" s="6" t="s">
         <v>20</v>
       </c>
@@ -14426,7 +14426,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="180" spans="1:17">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A180" s="6" t="s">
         <v>20</v>
       </c>
@@ -14479,7 +14479,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="181" spans="1:17">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A181" s="6" t="s">
         <v>20</v>
       </c>
@@ -14532,7 +14532,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="182" spans="1:17">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A182" s="6" t="s">
         <v>20</v>
       </c>
@@ -14585,7 +14585,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="183" spans="1:17">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A183" s="6" t="s">
         <v>20</v>
       </c>
@@ -14638,7 +14638,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="184" spans="1:17">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A184" s="6" t="s">
         <v>20</v>
       </c>
@@ -14691,7 +14691,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="185" spans="1:17">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A185" s="6" t="s">
         <v>20</v>
       </c>
@@ -14744,7 +14744,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="186" spans="1:17">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A186" s="6" t="s">
         <v>20</v>
       </c>
@@ -14797,7 +14797,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="187" spans="1:17">
+    <row r="187" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A187" s="6" t="s">
         <v>20</v>
       </c>
@@ -14850,7 +14850,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="188" spans="1:17">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A188" s="6" t="s">
         <v>20</v>
       </c>
@@ -14903,7 +14903,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="189" spans="1:17">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
         <v>20</v>
       </c>
@@ -14956,7 +14956,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="190" spans="1:17">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190" s="6" t="s">
         <v>20</v>
       </c>
@@ -15009,7 +15009,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="191" spans="1:17">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191" s="6" t="s">
         <v>20</v>
       </c>
@@ -15062,7 +15062,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="192" spans="1:17">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192" s="6" t="s">
         <v>20</v>
       </c>
@@ -15115,7 +15115,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="193" spans="1:17">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="6" t="s">
         <v>20</v>
       </c>
@@ -15168,7 +15168,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="194" spans="1:17">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="6" t="s">
         <v>20</v>
       </c>
@@ -15221,7 +15221,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="195" spans="1:17">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="6" t="s">
         <v>20</v>
       </c>
@@ -15274,7 +15274,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="196" spans="1:17">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="6" t="s">
         <v>20</v>
       </c>
@@ -15327,7 +15327,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="197" spans="1:17">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="6" t="s">
         <v>20</v>
       </c>
@@ -15380,7 +15380,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="198" spans="1:17">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="6" t="s">
         <v>20</v>
       </c>
@@ -15433,7 +15433,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="199" spans="1:17">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="6" t="s">
         <v>20</v>
       </c>
@@ -15486,7 +15486,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="200" spans="1:17">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="6" t="s">
         <v>20</v>
       </c>
@@ -15539,7 +15539,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="201" spans="1:17">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A201" s="6" t="s">
         <v>20</v>
       </c>
@@ -15592,7 +15592,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="202" spans="1:17">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A202" s="6" t="s">
         <v>20</v>
       </c>
@@ -15645,7 +15645,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="203" spans="1:17">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A203" s="6" t="s">
         <v>20</v>
       </c>
@@ -15698,7 +15698,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="204" spans="1:17">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A204" s="6" t="s">
         <v>20</v>
       </c>
@@ -15751,7 +15751,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="205" spans="1:17">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A205" s="6" t="s">
         <v>20</v>
       </c>
@@ -15804,7 +15804,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="206" spans="1:17">
+    <row r="206" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A206" s="6" t="s">
         <v>20</v>
       </c>
@@ -15857,7 +15857,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="207" spans="1:17">
+    <row r="207" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A207" s="6" t="s">
         <v>20</v>
       </c>
@@ -15910,7 +15910,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="208" spans="1:17">
+    <row r="208" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A208" s="6" t="s">
         <v>20</v>
       </c>
@@ -15963,7 +15963,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="209" spans="1:17">
+    <row r="209" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A209" s="6" t="s">
         <v>20</v>
       </c>
@@ -16016,7 +16016,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="210" spans="1:17">
+    <row r="210" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A210" s="6" t="s">
         <v>20</v>
       </c>
@@ -16069,7 +16069,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="211" spans="1:17">
+    <row r="211" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A211" s="6" t="s">
         <v>20</v>
       </c>
@@ -16122,7 +16122,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="212" spans="1:17">
+    <row r="212" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A212" s="6" t="s">
         <v>20</v>
       </c>
@@ -16175,7 +16175,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="213" spans="1:17">
+    <row r="213" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A213" s="6" t="s">
         <v>20</v>
       </c>
@@ -16228,7 +16228,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="214" spans="1:17">
+    <row r="214" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A214" s="6" t="s">
         <v>20</v>
       </c>
@@ -16281,7 +16281,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="215" spans="1:17">
+    <row r="215" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A215" s="6" t="s">
         <v>20</v>
       </c>
@@ -16334,7 +16334,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="216" spans="1:17">
+    <row r="216" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A216" s="6" t="s">
         <v>20</v>
       </c>
@@ -16387,7 +16387,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="217" spans="1:17">
+    <row r="217" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A217" s="6" t="s">
         <v>20</v>
       </c>
@@ -16440,7 +16440,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="218" spans="1:17">
+    <row r="218" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A218" s="6" t="s">
         <v>20</v>
       </c>
@@ -16493,7 +16493,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="219" spans="1:17">
+    <row r="219" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A219" s="6" t="s">
         <v>20</v>
       </c>
@@ -16546,7 +16546,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="220" spans="1:17">
+    <row r="220" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A220" s="6" t="s">
         <v>20</v>
       </c>
@@ -16599,7 +16599,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="221" spans="1:17">
+    <row r="221" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A221" s="6" t="s">
         <v>20</v>
       </c>
@@ -16652,7 +16652,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="222" spans="1:17">
+    <row r="222" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A222" s="6" t="s">
         <v>20</v>
       </c>
@@ -16705,7 +16705,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="223" spans="1:17">
+    <row r="223" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A223" s="6" t="s">
         <v>20</v>
       </c>
@@ -16758,7 +16758,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="224" spans="1:17">
+    <row r="224" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A224" s="6" t="s">
         <v>20</v>
       </c>
@@ -16811,7 +16811,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="225" spans="1:17">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A225" s="6" t="s">
         <v>20</v>
       </c>
@@ -16864,7 +16864,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="226" spans="1:17">
+    <row r="226" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A226" s="6" t="s">
         <v>20</v>
       </c>
@@ -16917,7 +16917,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="227" spans="1:17">
+    <row r="227" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A227" s="6" t="s">
         <v>20</v>
       </c>
@@ -16970,7 +16970,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="228" spans="1:17">
+    <row r="228" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A228" s="6" t="s">
         <v>20</v>
       </c>
@@ -17023,7 +17023,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="229" spans="1:17">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A229" s="6" t="s">
         <v>20</v>
       </c>
@@ -17076,7 +17076,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="230" spans="1:17">
+    <row r="230" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A230" s="6" t="s">
         <v>20</v>
       </c>
@@ -17129,7 +17129,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="231" spans="1:17">
+    <row r="231" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A231" s="6" t="s">
         <v>20</v>
       </c>
@@ -17182,7 +17182,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="232" spans="1:17">
+    <row r="232" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A232" s="6" t="s">
         <v>20</v>
       </c>
@@ -17235,7 +17235,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="233" spans="1:17">
+    <row r="233" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A233" s="6" t="s">
         <v>20</v>
       </c>
@@ -17288,7 +17288,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="234" spans="1:17">
+    <row r="234" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A234" s="6" t="s">
         <v>20</v>
       </c>
@@ -17341,7 +17341,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="235" spans="1:17">
+    <row r="235" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A235" s="6" t="s">
         <v>20</v>
       </c>
@@ -17394,7 +17394,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="236" spans="1:17">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A236" s="6" t="s">
         <v>20</v>
       </c>
@@ -17447,7 +17447,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="237" spans="1:17">
+    <row r="237" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A237" s="6" t="s">
         <v>20</v>
       </c>
@@ -17500,7 +17500,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="238" spans="1:17">
+    <row r="238" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A238" s="6" t="s">
         <v>20</v>
       </c>
@@ -17553,7 +17553,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="239" spans="1:17">
+    <row r="239" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A239" s="6" t="s">
         <v>20</v>
       </c>
@@ -17606,7 +17606,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="240" spans="1:17">
+    <row r="240" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A240" s="6" t="s">
         <v>20</v>
       </c>
@@ -17659,7 +17659,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="241" spans="1:17">
+    <row r="241" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A241" s="6" t="s">
         <v>20</v>
       </c>
@@ -17712,7 +17712,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="242" spans="1:17">
+    <row r="242" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A242" s="6" t="s">
         <v>20</v>
       </c>
@@ -17765,7 +17765,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="243" spans="1:17">
+    <row r="243" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A243" s="6" t="s">
         <v>20</v>
       </c>
@@ -17818,7 +17818,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="244" spans="1:17">
+    <row r="244" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A244" s="6" t="s">
         <v>20</v>
       </c>
@@ -17871,7 +17871,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="245" spans="1:17">
+    <row r="245" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A245" s="6" t="s">
         <v>20</v>
       </c>
@@ -17924,7 +17924,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="246" spans="1:17">
+    <row r="246" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A246" s="6" t="s">
         <v>20</v>
       </c>
@@ -17977,7 +17977,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="247" spans="1:17">
+    <row r="247" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A247" s="6" t="s">
         <v>20</v>
       </c>
@@ -18030,7 +18030,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="248" spans="1:17">
+    <row r="248" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A248" s="6" t="s">
         <v>20</v>
       </c>
@@ -18083,7 +18083,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="249" spans="1:17">
+    <row r="249" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A249" s="6" t="s">
         <v>20</v>
       </c>
@@ -18136,7 +18136,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="250" spans="1:17">
+    <row r="250" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A250" s="6" t="s">
         <v>20</v>
       </c>
@@ -18189,7 +18189,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="251" spans="1:17">
+    <row r="251" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A251" s="6" t="s">
         <v>20</v>
       </c>
@@ -18242,7 +18242,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="252" spans="1:17">
+    <row r="252" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A252" s="6" t="s">
         <v>20</v>
       </c>
@@ -18295,7 +18295,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="253" spans="1:17">
+    <row r="253" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A253" s="6" t="s">
         <v>20</v>
       </c>
@@ -18348,7 +18348,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="254" spans="1:17">
+    <row r="254" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A254" s="6" t="s">
         <v>20</v>
       </c>
@@ -18401,7 +18401,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="255" spans="1:17">
+    <row r="255" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A255" s="6" t="s">
         <v>20</v>
       </c>
@@ -18454,7 +18454,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="256" spans="1:17">
+    <row r="256" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A256" s="6" t="s">
         <v>20</v>
       </c>
@@ -18507,7 +18507,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="257" spans="1:17">
+    <row r="257" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A257" s="6" t="s">
         <v>20</v>
       </c>
@@ -18560,7 +18560,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="258" spans="1:17">
+    <row r="258" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A258" s="6" t="s">
         <v>20</v>
       </c>
@@ -18613,7 +18613,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="259" spans="1:17">
+    <row r="259" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A259" s="6" t="s">
         <v>20</v>
       </c>
@@ -18666,7 +18666,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="260" spans="1:17">
+    <row r="260" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A260" s="6" t="s">
         <v>20</v>
       </c>
@@ -18719,7 +18719,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="261" spans="1:17">
+    <row r="261" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A261" s="6" t="s">
         <v>20</v>
       </c>
@@ -18772,7 +18772,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="262" spans="1:17">
+    <row r="262" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A262" s="6" t="s">
         <v>20</v>
       </c>
@@ -18825,7 +18825,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="263" spans="1:17">
+    <row r="263" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A263" s="6" t="s">
         <v>20</v>
       </c>
@@ -18878,7 +18878,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="264" spans="1:17">
+    <row r="264" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A264" s="6" t="s">
         <v>20</v>
       </c>
@@ -18931,7 +18931,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="265" spans="1:17">
+    <row r="265" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A265" s="6" t="s">
         <v>20</v>
       </c>
@@ -18984,7 +18984,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="266" spans="1:17">
+    <row r="266" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A266" s="6" t="s">
         <v>20</v>
       </c>
@@ -19037,7 +19037,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="267" spans="1:17">
+    <row r="267" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A267" s="6" t="s">
         <v>20</v>
       </c>
@@ -19090,7 +19090,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="268" spans="1:17">
+    <row r="268" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A268" s="6" t="s">
         <v>20</v>
       </c>
@@ -19143,7 +19143,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="269" spans="1:17">
+    <row r="269" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A269" s="6" t="s">
         <v>20</v>
       </c>
@@ -19196,7 +19196,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="270" spans="1:17">
+    <row r="270" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A270" s="6" t="s">
         <v>20</v>
       </c>
@@ -19249,7 +19249,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="271" spans="1:17">
+    <row r="271" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A271" s="6" t="s">
         <v>20</v>
       </c>
@@ -19302,7 +19302,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="272" spans="1:17">
+    <row r="272" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A272" s="6" t="s">
         <v>20</v>
       </c>
@@ -19355,7 +19355,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="273" spans="1:17">
+    <row r="273" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A273" s="6" t="s">
         <v>20</v>
       </c>
@@ -19408,7 +19408,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="274" spans="1:17">
+    <row r="274" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A274" s="6" t="s">
         <v>20</v>
       </c>
@@ -19461,7 +19461,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="275" spans="1:17">
+    <row r="275" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A275" s="6" t="s">
         <v>20</v>
       </c>
@@ -19514,7 +19514,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="276" spans="1:17">
+    <row r="276" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A276" s="6" t="s">
         <v>20</v>
       </c>
@@ -19567,7 +19567,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="277" spans="1:17">
+    <row r="277" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A277" s="6" t="s">
         <v>20</v>
       </c>
@@ -19620,7 +19620,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="278" spans="1:17">
+    <row r="278" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A278" s="6" t="s">
         <v>20</v>
       </c>
@@ -19673,7 +19673,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="279" spans="1:17">
+    <row r="279" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A279" s="6" t="s">
         <v>20</v>
       </c>
@@ -19726,7 +19726,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="280" spans="1:17">
+    <row r="280" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A280" s="6" t="s">
         <v>20</v>
       </c>
@@ -19779,7 +19779,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="281" spans="1:17">
+    <row r="281" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A281" s="6" t="s">
         <v>20</v>
       </c>
@@ -19832,7 +19832,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="282" spans="1:17">
+    <row r="282" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A282" s="6" t="s">
         <v>20</v>
       </c>
@@ -19885,7 +19885,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="283" spans="1:17">
+    <row r="283" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A283" s="6" t="s">
         <v>20</v>
       </c>
@@ -19938,7 +19938,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="284" spans="1:17">
+    <row r="284" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A284" s="6" t="s">
         <v>20</v>
       </c>
@@ -19991,7 +19991,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="285" spans="1:17">
+    <row r="285" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A285" s="6" t="s">
         <v>20</v>
       </c>
@@ -20044,7 +20044,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="286" spans="1:17">
+    <row r="286" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A286" s="6" t="s">
         <v>20</v>
       </c>
@@ -20097,7 +20097,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="287" spans="1:17">
+    <row r="287" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A287" s="6" t="s">
         <v>20</v>
       </c>
@@ -20150,7 +20150,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="288" spans="1:17">
+    <row r="288" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A288" s="6" t="s">
         <v>20</v>
       </c>
@@ -20203,7 +20203,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="289" spans="1:17">
+    <row r="289" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A289" s="6" t="s">
         <v>20</v>
       </c>
@@ -20256,7 +20256,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="290" spans="1:17">
+    <row r="290" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A290" s="6" t="s">
         <v>20</v>
       </c>
@@ -20309,7 +20309,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="291" spans="1:17">
+    <row r="291" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A291" s="6" t="s">
         <v>20</v>
       </c>
@@ -20362,7 +20362,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="292" spans="1:17">
+    <row r="292" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A292" s="6" t="s">
         <v>20</v>
       </c>
@@ -20415,7 +20415,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="293" spans="1:17">
+    <row r="293" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A293" s="6" t="s">
         <v>20</v>
       </c>
@@ -20468,7 +20468,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="294" spans="1:17">
+    <row r="294" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A294" s="6" t="s">
         <v>20</v>
       </c>
@@ -20521,7 +20521,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="295" spans="1:17">
+    <row r="295" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A295" s="6" t="s">
         <v>20</v>
       </c>
@@ -20574,7 +20574,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="296" spans="1:17">
+    <row r="296" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A296" s="6" t="s">
         <v>20</v>
       </c>
@@ -20627,7 +20627,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="297" spans="1:17">
+    <row r="297" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A297" s="6" t="s">
         <v>20</v>
       </c>
@@ -20680,7 +20680,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="298" spans="1:17">
+    <row r="298" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A298" s="6" t="s">
         <v>20</v>
       </c>
@@ -20733,7 +20733,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="299" spans="1:17">
+    <row r="299" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A299" s="6" t="s">
         <v>20</v>
       </c>
@@ -20786,7 +20786,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="300" spans="1:17">
+    <row r="300" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A300" s="6" t="s">
         <v>20</v>
       </c>
@@ -20839,7 +20839,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="301" spans="1:17">
+    <row r="301" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A301" s="6" t="s">
         <v>20</v>
       </c>
@@ -20892,7 +20892,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="302" spans="1:17">
+    <row r="302" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A302" s="6" t="s">
         <v>20</v>
       </c>
@@ -20945,7 +20945,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="303" spans="1:17">
+    <row r="303" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A303" s="6" t="s">
         <v>20</v>
       </c>
@@ -20998,7 +20998,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="304" spans="1:17">
+    <row r="304" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A304" s="6" t="s">
         <v>20</v>
       </c>
@@ -21051,7 +21051,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="305" spans="1:17">
+    <row r="305" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A305" s="6" t="s">
         <v>20</v>
       </c>
@@ -21104,7 +21104,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="306" spans="1:17">
+    <row r="306" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A306" s="6" t="s">
         <v>20</v>
       </c>
@@ -21157,7 +21157,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="307" spans="1:17">
+    <row r="307" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A307" s="6" t="s">
         <v>20</v>
       </c>
@@ -21210,7 +21210,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="308" spans="1:17">
+    <row r="308" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A308" s="6" t="s">
         <v>20</v>
       </c>
@@ -21263,7 +21263,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="309" spans="1:17">
+    <row r="309" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A309" s="6" t="s">
         <v>20</v>
       </c>
@@ -21316,7 +21316,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="310" spans="1:17">
+    <row r="310" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A310" s="6" t="s">
         <v>20</v>
       </c>
@@ -21369,7 +21369,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="311" spans="1:17">
+    <row r="311" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A311" s="6" t="s">
         <v>20</v>
       </c>
@@ -21422,7 +21422,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="312" spans="1:17">
+    <row r="312" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A312" s="6" t="s">
         <v>20</v>
       </c>
@@ -21475,7 +21475,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="313" spans="1:17">
+    <row r="313" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A313" s="6" t="s">
         <v>20</v>
       </c>
@@ -21528,7 +21528,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="314" spans="1:17">
+    <row r="314" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A314" s="6" t="s">
         <v>20</v>
       </c>
@@ -21581,7 +21581,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="315" spans="1:17">
+    <row r="315" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A315" s="6" t="s">
         <v>20</v>
       </c>
@@ -21634,7 +21634,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="316" spans="1:17">
+    <row r="316" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A316" s="6" t="s">
         <v>20</v>
       </c>
@@ -21687,7 +21687,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="317" spans="1:17">
+    <row r="317" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A317" s="6" t="s">
         <v>20</v>
       </c>
@@ -21740,7 +21740,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="318" spans="1:17">
+    <row r="318" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A318" s="6" t="s">
         <v>20</v>
       </c>
@@ -21793,7 +21793,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="319" spans="1:17">
+    <row r="319" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A319" s="6" t="s">
         <v>20</v>
       </c>
@@ -21846,7 +21846,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="320" spans="1:17">
+    <row r="320" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A320" s="6" t="s">
         <v>20</v>
       </c>
@@ -21899,7 +21899,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="321" spans="1:17">
+    <row r="321" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A321" s="6" t="s">
         <v>20</v>
       </c>
@@ -21952,7 +21952,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="322" spans="1:17">
+    <row r="322" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A322" s="6" t="s">
         <v>20</v>
       </c>
@@ -22005,7 +22005,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="323" spans="1:17">
+    <row r="323" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A323" s="6" t="s">
         <v>20</v>
       </c>
@@ -22058,7 +22058,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="324" spans="1:17">
+    <row r="324" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A324" s="6" t="s">
         <v>20</v>
       </c>
@@ -22111,7 +22111,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="325" spans="1:17">
+    <row r="325" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A325" s="6" t="s">
         <v>20</v>
       </c>
@@ -22164,7 +22164,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="326" spans="1:17">
+    <row r="326" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A326" s="6" t="s">
         <v>20</v>
       </c>
@@ -22217,7 +22217,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="327" spans="1:17">
+    <row r="327" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A327" s="6" t="s">
         <v>20</v>
       </c>
@@ -22270,7 +22270,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="328" spans="1:17">
+    <row r="328" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A328" s="6" t="s">
         <v>20</v>
       </c>
@@ -22323,7 +22323,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="329" spans="1:17">
+    <row r="329" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A329" s="6" t="s">
         <v>20</v>
       </c>
@@ -22376,7 +22376,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="330" spans="1:17">
+    <row r="330" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A330" s="6" t="s">
         <v>20</v>
       </c>
@@ -22429,7 +22429,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="331" spans="1:17">
+    <row r="331" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A331" s="6" t="s">
         <v>20</v>
       </c>
@@ -22482,7 +22482,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="332" spans="1:17">
+    <row r="332" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A332" s="6" t="s">
         <v>20</v>
       </c>
@@ -22535,7 +22535,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="333" spans="1:17">
+    <row r="333" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A333" s="6" t="s">
         <v>20</v>
       </c>
@@ -22588,7 +22588,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="334" spans="1:17">
+    <row r="334" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A334" s="6" t="s">
         <v>20</v>
       </c>
@@ -22641,7 +22641,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="335" spans="1:17">
+    <row r="335" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A335" s="6" t="s">
         <v>20</v>
       </c>
@@ -22694,7 +22694,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="336" spans="1:17">
+    <row r="336" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A336" s="6" t="s">
         <v>20</v>
       </c>
@@ -22747,7 +22747,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="337" spans="1:17">
+    <row r="337" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A337" s="6" t="s">
         <v>20</v>
       </c>
@@ -22800,7 +22800,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="338" spans="1:17">
+    <row r="338" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A338" s="6" t="s">
         <v>20</v>
       </c>
@@ -22853,7 +22853,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="339" spans="1:17">
+    <row r="339" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A339" s="6" t="s">
         <v>20</v>
       </c>
@@ -22906,7 +22906,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="340" spans="1:17">
+    <row r="340" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A340" s="6" t="s">
         <v>20</v>
       </c>
@@ -22959,7 +22959,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="341" spans="1:17">
+    <row r="341" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A341" s="6" t="s">
         <v>20</v>
       </c>
@@ -23012,7 +23012,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="342" spans="1:17">
+    <row r="342" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A342" s="6" t="s">
         <v>20</v>
       </c>
@@ -23065,7 +23065,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="343" spans="1:17">
+    <row r="343" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A343" s="6" t="s">
         <v>20</v>
       </c>
@@ -23118,7 +23118,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="344" spans="1:17">
+    <row r="344" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A344" s="6" t="s">
         <v>20</v>
       </c>
@@ -23171,7 +23171,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="345" spans="1:17">
+    <row r="345" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A345" s="6" t="s">
         <v>20</v>
       </c>
@@ -23224,7 +23224,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="346" spans="1:17">
+    <row r="346" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A346" s="6" t="s">
         <v>20</v>
       </c>
@@ -23277,7 +23277,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="347" spans="1:17">
+    <row r="347" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A347" s="6" t="s">
         <v>20</v>
       </c>
@@ -23330,7 +23330,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="348" spans="1:17">
+    <row r="348" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A348" s="6" t="s">
         <v>20</v>
       </c>
@@ -23383,7 +23383,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="349" spans="1:17">
+    <row r="349" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A349" s="6" t="s">
         <v>20</v>
       </c>
@@ -23436,7 +23436,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="350" spans="1:17">
+    <row r="350" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A350" s="6" t="s">
         <v>20</v>
       </c>
@@ -23489,7 +23489,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="351" spans="1:17">
+    <row r="351" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A351" s="6" t="s">
         <v>20</v>
       </c>
@@ -23542,7 +23542,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="352" spans="1:17">
+    <row r="352" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A352" s="6" t="s">
         <v>20</v>
       </c>
@@ -23595,7 +23595,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="353" spans="1:17">
+    <row r="353" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A353" s="6" t="s">
         <v>20</v>
       </c>
@@ -23648,7 +23648,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="354" spans="1:17">
+    <row r="354" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A354" s="6" t="s">
         <v>20</v>
       </c>
@@ -23701,7 +23701,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="355" spans="1:17">
+    <row r="355" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A355" s="6" t="s">
         <v>20</v>
       </c>
@@ -23754,7 +23754,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="356" spans="1:17">
+    <row r="356" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A356" s="6" t="s">
         <v>20</v>
       </c>
@@ -23807,7 +23807,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="357" spans="1:17">
+    <row r="357" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A357" s="6" t="s">
         <v>20</v>
       </c>
@@ -23860,7 +23860,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="358" spans="1:17">
+    <row r="358" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A358" s="6" t="s">
         <v>20</v>
       </c>
@@ -23913,7 +23913,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="359" spans="1:17">
+    <row r="359" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A359" s="6" t="s">
         <v>20</v>
       </c>
@@ -23966,7 +23966,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="360" spans="1:17">
+    <row r="360" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A360" s="6" t="s">
         <v>20</v>
       </c>
@@ -24019,7 +24019,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="361" spans="1:17">
+    <row r="361" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A361" s="6" t="s">
         <v>20</v>
       </c>
@@ -24072,7 +24072,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="362" spans="1:17">
+    <row r="362" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A362" s="6" t="s">
         <v>20</v>
       </c>
@@ -24125,7 +24125,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="363" spans="1:17">
+    <row r="363" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A363" s="6" t="s">
         <v>20</v>
       </c>
@@ -24178,7 +24178,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="364" spans="1:17">
+    <row r="364" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A364" s="6" t="s">
         <v>20</v>
       </c>
@@ -24231,7 +24231,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="365" spans="1:17">
+    <row r="365" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A365" s="6" t="s">
         <v>20</v>
       </c>
@@ -24284,7 +24284,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="366" spans="1:17">
+    <row r="366" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A366" s="6" t="s">
         <v>20</v>
       </c>
@@ -24337,7 +24337,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="367" spans="1:17">
+    <row r="367" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A367" s="6" t="s">
         <v>20</v>
       </c>
@@ -24390,7 +24390,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="368" spans="1:17">
+    <row r="368" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A368" s="6" t="s">
         <v>20</v>
       </c>
@@ -24443,7 +24443,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="369" spans="1:17">
+    <row r="369" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A369" s="6" t="s">
         <v>20</v>
       </c>
@@ -24496,7 +24496,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="370" spans="1:17">
+    <row r="370" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A370" s="6" t="s">
         <v>20</v>
       </c>
@@ -24549,7 +24549,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="371" spans="1:17">
+    <row r="371" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A371" s="6" t="s">
         <v>20</v>
       </c>
@@ -24602,7 +24602,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="372" spans="1:17">
+    <row r="372" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A372" s="6" t="s">
         <v>20</v>
       </c>
@@ -24655,7 +24655,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="373" spans="1:17">
+    <row r="373" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A373" s="6" t="s">
         <v>20</v>
       </c>
@@ -24708,7 +24708,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="374" spans="1:17">
+    <row r="374" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A374" s="6" t="s">
         <v>20</v>
       </c>
@@ -24761,7 +24761,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="375" spans="1:17">
+    <row r="375" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A375" s="6" t="s">
         <v>20</v>
       </c>
@@ -24814,7 +24814,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="376" spans="1:17">
+    <row r="376" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A376" s="6" t="s">
         <v>20</v>
       </c>
@@ -24867,7 +24867,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="377" spans="1:17">
+    <row r="377" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A377" s="6" t="s">
         <v>20</v>
       </c>
@@ -24920,7 +24920,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="378" spans="1:17">
+    <row r="378" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A378" s="6" t="s">
         <v>20</v>
       </c>
@@ -24973,7 +24973,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="379" spans="1:17">
+    <row r="379" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A379" s="6" t="s">
         <v>20</v>
       </c>
@@ -25026,7 +25026,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="380" spans="1:17">
+    <row r="380" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A380" s="6" t="s">
         <v>20</v>
       </c>
@@ -25079,7 +25079,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="381" spans="1:17">
+    <row r="381" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A381" s="6" t="s">
         <v>20</v>
       </c>
@@ -25132,7 +25132,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="382" spans="1:17">
+    <row r="382" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A382" s="6" t="s">
         <v>20</v>
       </c>
@@ -25185,7 +25185,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="383" spans="1:17">
+    <row r="383" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A383" s="6" t="s">
         <v>20</v>
       </c>
@@ -25238,7 +25238,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="384" spans="1:17">
+    <row r="384" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A384" s="6" t="s">
         <v>20</v>
       </c>
@@ -25291,7 +25291,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="385" spans="1:17">
+    <row r="385" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A385" s="6" t="s">
         <v>20</v>
       </c>
@@ -25344,7 +25344,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="386" spans="1:17">
+    <row r="386" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A386" s="6" t="s">
         <v>20</v>
       </c>
@@ -25397,7 +25397,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="387" spans="1:17">
+    <row r="387" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A387" s="6" t="s">
         <v>20</v>
       </c>
@@ -25450,7 +25450,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="388" spans="1:17">
+    <row r="388" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A388" s="6" t="s">
         <v>20</v>
       </c>
@@ -25503,7 +25503,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="389" spans="1:17">
+    <row r="389" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A389" s="6" t="s">
         <v>20</v>
       </c>
@@ -25556,7 +25556,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="390" spans="1:17">
+    <row r="390" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A390" s="6" t="s">
         <v>20</v>
       </c>
@@ -25609,7 +25609,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="391" spans="1:17">
+    <row r="391" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A391" s="6" t="s">
         <v>20</v>
       </c>
@@ -25662,7 +25662,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="392" spans="1:17">
+    <row r="392" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A392" s="6" t="s">
         <v>20</v>
       </c>
@@ -25715,7 +25715,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="393" spans="1:17">
+    <row r="393" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A393" s="6" t="s">
         <v>20</v>
       </c>
@@ -25768,7 +25768,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="394" spans="1:17">
+    <row r="394" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A394" s="6" t="s">
         <v>20</v>
       </c>
@@ -25821,7 +25821,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="395" spans="1:17">
+    <row r="395" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A395" s="6" t="s">
         <v>20</v>
       </c>
@@ -25874,7 +25874,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="396" spans="1:17">
+    <row r="396" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A396" s="6" t="s">
         <v>20</v>
       </c>
@@ -25927,7 +25927,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="397" spans="1:17">
+    <row r="397" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A397" s="6" t="s">
         <v>20</v>
       </c>
@@ -25980,7 +25980,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="398" spans="1:17">
+    <row r="398" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A398" s="6" t="s">
         <v>20</v>
       </c>
@@ -26033,7 +26033,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="399" spans="1:17">
+    <row r="399" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A399" s="6" t="s">
         <v>20</v>
       </c>
@@ -26086,7 +26086,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="400" spans="1:17">
+    <row r="400" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A400" s="6" t="s">
         <v>20</v>
       </c>
@@ -26139,7 +26139,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="401" spans="1:17">
+    <row r="401" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A401" s="6" t="s">
         <v>20</v>
       </c>
@@ -26192,7 +26192,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="402" spans="1:17">
+    <row r="402" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A402" s="6" t="s">
         <v>20</v>
       </c>
@@ -26245,7 +26245,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="403" spans="1:17">
+    <row r="403" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A403" s="6" t="s">
         <v>20</v>
       </c>
@@ -26298,7 +26298,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="404" spans="1:17">
+    <row r="404" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A404" s="6" t="s">
         <v>20</v>
       </c>
@@ -26351,7 +26351,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="405" spans="1:17">
+    <row r="405" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A405" s="6" t="s">
         <v>20</v>
       </c>
@@ -26404,7 +26404,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="406" spans="1:17">
+    <row r="406" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A406" s="6" t="s">
         <v>20</v>
       </c>
@@ -26457,7 +26457,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="407" spans="1:17">
+    <row r="407" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A407" s="6" t="s">
         <v>20</v>
       </c>
@@ -26510,7 +26510,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="408" spans="1:17">
+    <row r="408" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A408" s="6" t="s">
         <v>20</v>
       </c>
@@ -26563,7 +26563,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="409" spans="1:17">
+    <row r="409" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A409" s="6" t="s">
         <v>20</v>
       </c>
@@ -26616,7 +26616,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="410" spans="1:17">
+    <row r="410" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A410" s="6" t="s">
         <v>20</v>
       </c>
@@ -26669,7 +26669,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="411" spans="1:17">
+    <row r="411" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A411" s="6" t="s">
         <v>20</v>
       </c>
@@ -26722,7 +26722,7 @@
         <v>1520</v>
       </c>
     </row>
-    <row r="412" spans="1:17">
+    <row r="412" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A412" s="6" t="s">
         <v>20</v>
       </c>
@@ -26789,12 +26789,7 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<SyracuseOfficeCustomData>{"createMode":"plain_doc","forceRefresh":"0"}</SyracuseOfficeCustomData>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -27076,7 +27071,12 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<SyracuseOfficeCustomData>{"createMode":"plain_doc","forceRefresh":"0"}</SyracuseOfficeCustomData>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -27093,17 +27093,47 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EDC6E94-DEF6-44D5-88D7-1A24FC258DF7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76AD796C-2652-4588-B29C-C1F0B889E6EA}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A1F794B-AC8B-48C2-8E03-4DE2CC746C9E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A1F794B-AC8B-48C2-8E03-4DE2CC746C9E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="8ff73537-c08d-4f8f-aeba-20b03f614348"/>
+    <ds:schemaRef ds:uri="22ffcb7a-b1bb-4c2a-b364-2b664037746d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76AD796C-2652-4588-B29C-C1F0B889E6EA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3EDC6E94-DEF6-44D5-88D7-1A24FC258DF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CC37542-CDFE-41EA-B8B1-BB979EE4C368}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CC37542-CDFE-41EA-B8B1-BB979EE4C368}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="22ffcb7a-b1bb-4c2a-b364-2b664037746d"/>
+    <ds:schemaRef ds:uri="8ff73537-c08d-4f8f-aeba-20b03f614348"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>